<commit_message>
Added support for OSPM model
</commit_message>
<xml_diff>
--- a/model_paths/model_paths_and_files.xlsx
+++ b/model_paths/model_paths_and_files.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Prog\NORTRIP-python\model_paths\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sindredenby/Documents/metrologisk/NORTRIP-python/model_paths/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A2AB80-403B-4DE8-B7C6-24B2A8EDA0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C7193E-3A11-4E40-8FC5-71E206011EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Filenames" sheetId="1" r:id="rId1"/>
@@ -86,9 +86,6 @@
     <t>C:\WORK\NORTRIP\NORTRIP\NORTRIP_model_public_v3_4\fortran\output\</t>
   </si>
   <si>
-    <t>C:\Prog\ospm\</t>
-  </si>
-  <si>
     <t>model_parameters/</t>
   </si>
   <si>
@@ -108,6 +105,9 @@
   </si>
   <si>
     <t>Comments</t>
+  </si>
+  <si>
+    <t>ospm/</t>
   </si>
 </sst>
 </file>
@@ -481,15 +481,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="95.28515625" customWidth="1"/>
-    <col min="3" max="3" width="58.7109375" customWidth="1"/>
-    <col min="4" max="4" width="42.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="95.33203125" customWidth="1"/>
+    <col min="3" max="3" width="58.6640625" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -497,50 +497,50 @@
         <v>5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -548,23 +548,23 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -572,7 +572,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -580,7 +580,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>

</xml_diff>